<commit_message>
docs: add EXPO_PROJECT_OVERVIEW docx and markdown overview for expo evaluation
</commit_message>
<xml_diff>
--- a/OA_MODELS_BENCHMARKS_AND_METRICS.xlsx
+++ b/OA_MODELS_BENCHMARKS_AND_METRICS.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f523a37c22dacd7e/Desktop/Projects/OA_NER Screening/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_907863AA71899F06691F5A6BF284BAA844C0A822" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C71DDB2-6C86-44EC-A478-D6D6E78504E2}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Executive Model Summary" sheetId="1" r:id="rId1"/>
@@ -13,7 +19,7 @@
     <sheet name="3. BMD &amp; X-Ray Models" sheetId="4" r:id="rId4"/>
     <sheet name="Cloud &amp; API Architecture" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -575,12 +581,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#,##0"/>
-    <numFmt numFmtId="165" formatCode="0.00%"/>
-  </numFmts>
-  <fonts count="7">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -703,13 +705,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -721,13 +723,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -765,7 +775,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -799,6 +809,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -833,9 +844,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1008,32 +1020,32 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
-    <col min="4" max="4" width="32.7109375" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" customWidth="1"/>
-    <col min="8" max="9" width="20.7109375" customWidth="1"/>
-    <col min="10" max="10" width="36.7109375" customWidth="1"/>
+    <col min="1" max="1" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="24.6640625" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="4" max="4" width="32.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="9" width="20.6640625" customWidth="1"/>
+    <col min="10" max="10" width="48.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1065,7 +1077,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
@@ -1082,22 +1094,22 @@
         <v>9580</v>
       </c>
       <c r="F5" s="7">
-        <v>0.8269</v>
+        <v>0.82689999999999997</v>
       </c>
       <c r="G5" s="7">
-        <v>0.8708</v>
+        <v>0.87080000000000002</v>
       </c>
       <c r="H5" s="7">
-        <v>0.8329</v>
+        <v>0.83289999999999997</v>
       </c>
       <c r="I5" s="7">
-        <v>0.8292</v>
+        <v>0.82920000000000005</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>17</v>
       </c>
@@ -1114,22 +1126,22 @@
         <v>125</v>
       </c>
       <c r="F6" s="7">
-        <v>0.744</v>
+        <v>0.74399999999999999</v>
       </c>
       <c r="G6" s="7">
-        <v>0.793</v>
+        <v>0.79300000000000004</v>
       </c>
       <c r="H6" s="7">
-        <v>0.7452</v>
+        <v>0.74519999999999997</v>
       </c>
       <c r="I6" s="7">
-        <v>0.7445000000000001</v>
+        <v>0.74450000000000005</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>22</v>
       </c>
@@ -1146,22 +1158,22 @@
         <v>540</v>
       </c>
       <c r="F7" s="7">
-        <v>0.8018999999999999</v>
+        <v>0.80189999999999995</v>
       </c>
       <c r="G7" s="7">
-        <v>0.841</v>
+        <v>0.84099999999999997</v>
       </c>
       <c r="H7" s="7">
-        <v>0.804</v>
+        <v>0.80400000000000005</v>
       </c>
       <c r="I7" s="7">
-        <v>0.798</v>
+        <v>0.79800000000000004</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>27</v>
       </c>
@@ -1178,22 +1190,22 @@
         <v>4200</v>
       </c>
       <c r="F8" s="7">
-        <v>0.864</v>
+        <v>0.86399999999999999</v>
       </c>
       <c r="G8" s="7">
-        <v>0.912</v>
+        <v>0.91200000000000003</v>
       </c>
       <c r="H8" s="7">
-        <v>0.868</v>
+        <v>0.86799999999999999</v>
       </c>
       <c r="I8" s="7">
-        <v>0.862</v>
+        <v>0.86199999999999999</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>32</v>
       </c>
@@ -1231,25 +1243,25 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E33"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.7109375" customWidth="1"/>
-    <col min="2" max="5" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" customWidth="1"/>
+    <col min="2" max="5" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>40</v>
       </c>
@@ -1257,23 +1269,23 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>42</v>
       </c>
       <c r="B5" s="7">
-        <v>0.8269</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+        <v>0.82689999999999997</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>43</v>
       </c>
       <c r="B6" s="7">
-        <v>0.8708</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
+        <v>0.87080000000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>44</v>
       </c>
@@ -1281,36 +1293,36 @@
         <v>9580</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>45</v>
       </c>
       <c r="B8" s="8">
-        <v>0.8329</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
+        <v>0.83289999999999997</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>46</v>
       </c>
       <c r="B9" s="8">
-        <v>0.8269</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
+        <v>0.82689999999999997</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>47</v>
       </c>
       <c r="B10" s="8">
-        <v>0.8292</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
+        <v>0.82920000000000005</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>49</v>
       </c>
@@ -1327,24 +1339,24 @@
         <v>53</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B14" s="8">
-        <v>0.8942</v>
+        <v>0.89419999999999999</v>
       </c>
       <c r="C14" s="8">
-        <v>0.8591</v>
+        <v>0.85909999999999997</v>
       </c>
       <c r="D14" s="8">
-        <v>0.8763</v>
+        <v>0.87629999999999997</v>
       </c>
       <c r="E14" s="6">
         <v>6835</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>55</v>
       </c>
@@ -1352,21 +1364,21 @@
         <v>0.6804</v>
       </c>
       <c r="C15" s="8">
-        <v>0.7468</v>
+        <v>0.74680000000000002</v>
       </c>
       <c r="D15" s="8">
-        <v>0.7121</v>
+        <v>0.71209999999999996</v>
       </c>
       <c r="E15" s="6">
         <v>2745</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
@@ -1377,7 +1389,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>60</v>
       </c>
@@ -1388,7 +1400,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>61</v>
       </c>
@@ -1399,12 +1411,12 @@
         <v>5872</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>63</v>
       </c>
@@ -1415,111 +1427,111 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>66</v>
       </c>
       <c r="B24" s="8">
-        <v>0.2735</v>
+        <v>0.27350000000000002</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>68</v>
       </c>
       <c r="B25" s="8">
-        <v>0.1403</v>
+        <v>0.14030000000000001</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>70</v>
       </c>
       <c r="B26" s="8">
-        <v>0.1247</v>
+        <v>0.12470000000000001</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>72</v>
       </c>
       <c r="B27" s="8">
-        <v>0.09329999999999999</v>
+        <v>9.3299999999999994E-2</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>74</v>
       </c>
       <c r="B28" s="8">
-        <v>0.053</v>
+        <v>5.2999999999999999E-2</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>76</v>
       </c>
       <c r="B29" s="8">
-        <v>0.0432</v>
+        <v>4.3200000000000002E-2</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>78</v>
       </c>
       <c r="B30" s="8">
-        <v>0.041</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>80</v>
       </c>
       <c r="B31" s="8">
-        <v>0.0401</v>
+        <v>4.0099999999999997E-2</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>82</v>
       </c>
       <c r="B32" s="8">
-        <v>0.0392</v>
+        <v>3.9199999999999999E-2</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>84</v>
       </c>
       <c r="B33" s="8">
-        <v>0.038</v>
+        <v>3.7999999999999999E-2</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>85</v>
@@ -1531,62 +1543,62 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.7109375" customWidth="1"/>
-    <col min="2" max="5" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" customWidth="1"/>
+    <col min="2" max="5" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>42</v>
       </c>
       <c r="B5" s="7">
-        <v>0.744</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+        <v>0.74399999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>47</v>
       </c>
       <c r="B6" s="7">
-        <v>0.7445000000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
+        <v>0.74450000000000005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>45</v>
       </c>
       <c r="B7" s="8">
-        <v>0.7452</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
+        <v>0.74519999999999997</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>89</v>
       </c>
       <c r="B8" s="8">
-        <v>0.744</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
+        <v>0.74399999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>90</v>
       </c>
@@ -1594,12 +1606,12 @@
         <v>125</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>92</v>
       </c>
@@ -1616,24 +1628,24 @@
         <v>94</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>95</v>
       </c>
       <c r="B13" s="8">
-        <v>0.9804</v>
+        <v>0.98040000000000005</v>
       </c>
       <c r="C13" s="8">
-        <v>0.9804</v>
+        <v>0.98040000000000005</v>
       </c>
       <c r="D13" s="8">
-        <v>0.9804</v>
+        <v>0.98040000000000005</v>
       </c>
       <c r="E13" s="6">
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>96</v>
       </c>
@@ -1650,7 +1662,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>97</v>
       </c>
@@ -1658,38 +1670,38 @@
         <v>0.6</v>
       </c>
       <c r="C15" s="8">
-        <v>0.5769</v>
+        <v>0.57689999999999997</v>
       </c>
       <c r="D15" s="8">
-        <v>0.5881999999999999</v>
+        <v>0.58819999999999995</v>
       </c>
       <c r="E15" s="6">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>98</v>
       </c>
       <c r="B16" s="8">
-        <v>0.4483</v>
+        <v>0.44829999999999998</v>
       </c>
       <c r="C16" s="8">
-        <v>0.4643</v>
+        <v>0.46429999999999999</v>
       </c>
       <c r="D16" s="8">
-        <v>0.4561</v>
+        <v>0.45610000000000001</v>
       </c>
       <c r="E16" s="6">
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>100</v>
       </c>
@@ -1703,7 +1715,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>104</v>
       </c>
@@ -1717,7 +1729,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>108</v>
       </c>
@@ -1731,7 +1743,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>112</v>
       </c>
@@ -1745,7 +1757,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>116</v>
       </c>
@@ -1765,48 +1777,48 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="4" width="38.7109375" customWidth="1"/>
+    <col min="1" max="1" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="24.6640625" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" customWidth="1"/>
+    <col min="4" max="4" width="38.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>123</v>
       </c>
       <c r="B5" s="7">
-        <v>0.8018999999999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>0.80189999999999995</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>124</v>
       </c>
       <c r="B6" s="7">
-        <v>0.7444</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+        <v>0.74439999999999995</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>125</v>
       </c>
@@ -1814,7 +1826,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>127</v>
       </c>
@@ -1822,28 +1834,28 @@
         <v>128</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>130</v>
       </c>
       <c r="B11" s="7">
-        <v>0.864</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
+        <v>0.86399999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>131</v>
       </c>
       <c r="B12" s="7">
-        <v>0.912</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
+        <v>0.91200000000000003</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>132</v>
       </c>
@@ -1851,7 +1863,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>134</v>
       </c>
@@ -1865,32 +1877,32 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" customWidth="1"/>
-    <col min="2" max="2" width="30.7109375" customWidth="1"/>
-    <col min="3" max="3" width="42.7109375" customWidth="1"/>
-    <col min="4" max="4" width="24.7109375" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" customWidth="1"/>
+    <col min="2" max="2" width="30.6640625" customWidth="1"/>
+    <col min="3" max="3" width="42.6640625" customWidth="1"/>
+    <col min="4" max="4" width="24.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>139</v>
       </c>
@@ -1904,7 +1916,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>143</v>
       </c>
@@ -1918,7 +1930,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>147</v>
       </c>
@@ -1932,7 +1944,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>150</v>
       </c>
@@ -1946,7 +1958,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>153</v>
       </c>
@@ -1960,7 +1972,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>156</v>
       </c>
@@ -1974,12 +1986,12 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>161</v>
       </c>
@@ -1993,7 +2005,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>165</v>
       </c>
@@ -2007,7 +2019,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>169</v>
       </c>
@@ -2021,7 +2033,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>172</v>
       </c>
@@ -2035,7 +2047,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>176</v>
       </c>
@@ -2049,7 +2061,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>180</v>
       </c>

</xml_diff>